<commit_message>
Improve live sheet detection (area-ranked contours) and sync scanner/project files for deployment
Co-authored-by: Junie <junie@jetbrains.com>
</commit_message>
<xml_diff>
--- a/batch_adrian.xlsx
+++ b/batch_adrian.xlsx
@@ -29,7 +29,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -38,7 +38,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
+        <fgColor rgb="00FF6B6B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFA500"/>
       </patternFill>
     </fill>
   </fills>
@@ -54,10 +59,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ3"/>
+  <dimension ref="A1:AR3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -469,6 +475,7 @@
     <col width="10" customWidth="1" min="41" max="41"/>
     <col width="10" customWidth="1" min="42" max="42"/>
     <col width="10" customWidth="1" min="43" max="43"/>
+    <col width="10" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -684,7 +691,12 @@
       </c>
       <c r="AQ1" s="1" t="inlineStr">
         <is>
-          <t>Flagged (low confidence)</t>
+          <t>Flagged Questions</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>Avg Confidence</t>
         </is>
       </c>
     </row>
@@ -693,74 +705,213 @@
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr"/>
-      <c r="C2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="n"/>
-      <c r="P2" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>4</v>
-      </c>
-      <c r="R2" t="n">
-        <v>4</v>
-      </c>
-      <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
-      <c r="U2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="V2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>Q1, Q2, Q3, Q4, Q5, Q6, Q7, Q8, Q12, Q13, Q17, Q18, Q19, Q20</t>
-        </is>
+          <t>Too few circles remain (5) after radius filtering.</t>
+        </is>
+      </c>
+      <c r="AR2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -768,130 +919,71 @@
         <v>2</v>
       </c>
       <c r="B3" t="inlineStr"/>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="N3" s="2" t="n"/>
+      <c r="O3" s="2" t="n"/>
+      <c r="P3" s="2" t="n"/>
+      <c r="Q3" s="2" t="n"/>
+      <c r="R3" s="2" t="n"/>
+      <c r="S3" s="2" t="n"/>
+      <c r="T3" s="2" t="n"/>
+      <c r="U3" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="V3" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="L3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="P3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="R3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="S3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="T3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="U3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="V3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="W3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="X3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AB3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AI3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AJ3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AK3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AO3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP3" s="2" t="n">
-        <v>2</v>
+      <c r="W3" s="2" t="n"/>
+      <c r="X3" s="2" t="n"/>
+      <c r="Y3" s="2" t="n"/>
+      <c r="Z3" s="2" t="n"/>
+      <c r="AA3" s="2" t="n"/>
+      <c r="AB3" s="2" t="n"/>
+      <c r="AC3" s="2" t="n"/>
+      <c r="AD3" s="2" t="n"/>
+      <c r="AE3" s="2" t="n"/>
+      <c r="AF3" s="2" t="n"/>
+      <c r="AG3" s="2" t="n"/>
+      <c r="AH3" s="2" t="n"/>
+      <c r="AI3" s="2" t="n"/>
+      <c r="AJ3" s="2" t="n"/>
+      <c r="AK3" s="2" t="n"/>
+      <c r="AL3" s="2" t="n"/>
+      <c r="AM3" s="2" t="n"/>
+      <c r="AN3" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP3" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
           <t>Q1, Q2, Q3, Q4, Q5, Q6, Q7, Q8, Q9, Q10, Q11, Q12, Q13, Q14, Q15, Q16, Q17, Q18, Q19, Q20, Q21, Q22, Q23, Q24, Q25, Q26, Q27, Q28, Q29, Q30, Q31, Q32, Q33, Q34, Q35, Q36, Q37, Q38, Q39, Q40</t>
         </is>
+      </c>
+      <c r="AR3" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>